<commit_message>
Eredivisie bijgewerkt 08-09-2026 12:01
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 September 2026 om 13:21</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 September 2026 om 12:01</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 September 2026 om 13:21</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 September 2026 om 12:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 10-09-2026 12:06
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 September 2026 om 12:12</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 September 2026 om 12:06</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
@@ -1169,14 +1169,14 @@
         <v>10</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
@@ -1191,29 +1191,29 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
         <v>5</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>60%</t>
         </is>
       </c>
     </row>
@@ -1232,48 +1232,48 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>40%</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C10" s="20" t="n">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D16" s="20" t="n">
         <v>1</v>
@@ -1532,7 +1532,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G16" s="21" t="n">
         <v>4</v>
@@ -1541,16 +1541,16 @@
         <v>5</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J16" s="23" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="K16" s="20" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 September 2026 om 12:12</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 September 2026 om 12:06</t>
         </is>
       </c>
     </row>
@@ -15974,9 +15974,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="R7" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="R7" s="39" t="inlineStr">
+        <is>
+          <t>1-0</t>
         </is>
       </c>
       <c r="S7" s="35" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 11-09-2026 12:05
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 September 2026 om 12:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 September 2026 om 12:05</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 September 2026 om 12:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 September 2026 om 12:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 12-09-2026 11:31
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 September 2026 om 12:05</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 September 2026 om 11:31</t>
         </is>
       </c>
     </row>
@@ -990,25 +990,25 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>5</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>83%</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>ADO Den Haag</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="C18" s="20" t="n">
@@ -1611,23 +1611,23 @@
         <v>0</v>
       </c>
       <c r="E18" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G18" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I18" s="20" t="n">
         <v>14</v>
       </c>
       <c r="J18" s="23" t="inlineStr">
         <is>
-          <t>-8</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
@@ -1642,11 +1642,11 @@
       </c>
       <c r="B19" s="26" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>ADO Den Haag</t>
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>0</v>
@@ -1655,20 +1655,20 @@
         <v>1</v>
       </c>
       <c r="F19" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G19" s="28" t="n">
         <v>1</v>
       </c>
       <c r="H19" s="27" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J19" s="29" t="inlineStr">
         <is>
-          <t>-9</t>
+          <t>-8</t>
         </is>
       </c>
       <c r="K19" s="27" t="inlineStr">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 September 2026 om 12:05</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 September 2026 om 11:31</t>
         </is>
       </c>
     </row>
@@ -15785,9 +15785,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="S5" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="S5" s="38" t="inlineStr">
+        <is>
+          <t>1-1</t>
         </is>
       </c>
     </row>
@@ -33729,13 +33729,13 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 14-09-2026 13:45
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 September 2026 om 12:36</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 September 2026 om 13:45</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -1005,14 +1005,14 @@
         <v>16</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>+11</t>
+          <t>+15</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -1027,14 +1027,14 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C4" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" s="10" t="n">
         <v>5</v>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>4</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>1</v>
@@ -1043,22 +1043,22 @@
         <v>0</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I4" s="10" t="n">
         <v>6</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>+12</t>
+          <t>+11</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>83%</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>Feyenoord Rotterdam</t>
         </is>
       </c>
       <c r="C5" s="10" t="n">
@@ -1078,23 +1078,23 @@
         <v>4</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+13</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
@@ -1109,38 +1109,38 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>11</v>
-      </c>
-      <c r="H6" s="10" t="n">
-        <v>13</v>
-      </c>
-      <c r="I6" s="10" t="n">
-        <v>7</v>
-      </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+6</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D14" s="20" t="n">
         <v>1</v>
@@ -1450,25 +1450,25 @@
         <v>2</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" s="21" t="n">
         <v>5</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="J14" s="20" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v>13</v>
+      </c>
+      <c r="J14" s="23" t="inlineStr">
+        <is>
+          <t>-3</t>
         </is>
       </c>
       <c r="K14" s="20" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>17%</t>
         </is>
       </c>
     </row>
@@ -1560,11 +1560,11 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>PEC Zwolle</t>
+          <t>SC Cambuur-Leeuwarden</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>1</v>
@@ -1573,25 +1573,25 @@
         <v>1</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G17" s="16" t="n">
         <v>4</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>-4</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="K17" s="15" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>17%</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>SC Cambuur-Leeuwarden</t>
+          <t>PEC Zwolle</t>
         </is>
       </c>
       <c r="C18" s="20" t="n">
@@ -1620,14 +1620,14 @@
         <v>4</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J18" s="23" t="inlineStr">
         <is>
-          <t>-9</t>
+          <t>-11</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 September 2026 om 12:36</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 September 2026 om 13:45</t>
         </is>
       </c>
     </row>
@@ -16506,9 +16506,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="H13" s="35" t="inlineStr">
+        <is>
+          <t>0-7</t>
         </is>
       </c>
       <c r="I13" s="34" t="inlineStr">
@@ -16648,9 +16648,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="Q14" s="34" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="Q14" s="38" t="inlineStr">
+        <is>
+          <t>4-1</t>
         </is>
       </c>
       <c r="R14" s="34" t="inlineStr">
@@ -16944,9 +16944,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="R17" s="34" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="R17" s="37" t="inlineStr">
+        <is>
+          <t>0-0</t>
         </is>
       </c>
       <c r="S17" s="34" t="inlineStr">
@@ -33725,21 +33725,21 @@
       </c>
       <c r="B5" s="45" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>+11</t>
+          <t>+15</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
@@ -33785,7 +33785,7 @@
         </is>
       </c>
       <c r="I6" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="20" t="n">
         <v>14</v>
@@ -33852,17 +33852,6 @@
         <is>
           <t>+51</t>
         </is>
-      </c>
-      <c r="H8" s="48" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="I8" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="20" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 15-09-2026 12:31
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 September 2026 om 13:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 September 2026 om 12:31</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 September 2026 om 13:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 September 2026 om 12:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 16-09-2026 12:29
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 September 2026 om 12:31</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 September 2026 om 12:29</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
@@ -1128,14 +1128,14 @@
         <v>13</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+12</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
@@ -1150,14 +1150,14 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>1</v>
@@ -1166,22 +1166,22 @@
         <v>1</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>+8</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
         </is>
       </c>
       <c r="C19" s="26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D19" s="26" t="n">
         <v>0</v>
@@ -1655,20 +1655,20 @@
         <v>2</v>
       </c>
       <c r="F19" s="26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G19" s="27" t="n">
         <v>2</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I19" s="26" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="J19" s="28" t="inlineStr">
         <is>
-          <t>-9</t>
+          <t>-13</t>
         </is>
       </c>
       <c r="K19" s="26" t="inlineStr">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 September 2026 om 12:31</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 September 2026 om 12:29</t>
         </is>
       </c>
     </row>
@@ -15688,9 +15688,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="S4" s="34" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="S4" s="38" t="inlineStr">
+        <is>
+          <t>5-1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 17-09-2026 12:28
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 September 2026 om 12:29</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 September 2026 om 12:28</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 September 2026 om 12:29</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 September 2026 om 12:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 18-09-2026 12:07
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 September 2026 om 12:28</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 September 2026 om 12:07</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 September 2026 om 12:28</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 September 2026 om 12:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 19-09-2026 11:50
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -315,7 +315,7 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -330,10 +330,10 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -382,7 +382,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 September 2026 om 12:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 September 2026 om 11:50</t>
         </is>
       </c>
     </row>
@@ -1191,38 +1191,38 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H8" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="I8" s="10" t="n">
-        <v>7</v>
-      </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>+6</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>43%</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
@@ -1251,14 +1251,14 @@
         <v>10</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>+6</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
@@ -1273,38 +1273,38 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C10" s="20" t="n">
         <v>6</v>
       </c>
       <c r="D10" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10" s="20" t="n">
-        <v>1</v>
-      </c>
       <c r="G10" s="21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I10" s="20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J10" s="22" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>FC Groningen</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
@@ -1324,23 +1324,23 @@
         <v>2</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I11" s="15" t="n">
         <v>13</v>
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
@@ -1379,7 +1379,7 @@
       <c r="I12" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -1420,7 +1420,7 @@
       <c r="I13" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -1461,7 +1461,7 @@
       <c r="I14" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -1502,7 +1502,7 @@
       <c r="I15" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -1543,7 +1543,7 @@
       <c r="I16" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -1584,7 +1584,7 @@
       <c r="I17" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="C18" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D18" s="20" t="n">
         <v>1</v>
@@ -1614,7 +1614,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G18" s="21" t="n">
         <v>4</v>
@@ -1623,16 +1623,16 @@
         <v>6</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>17</v>
-      </c>
-      <c r="J18" s="23" t="inlineStr">
-        <is>
-          <t>-11</t>
+        <v>20</v>
+      </c>
+      <c r="J18" s="22" t="inlineStr">
+        <is>
+          <t>-14</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>14%</t>
         </is>
       </c>
     </row>
@@ -3984,7 +3984,7 @@
       <c r="I9" s="15" t="n">
         <v>37</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+3</t>
         </is>
@@ -4025,7 +4025,7 @@
       <c r="I10" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="40" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -4066,7 +4066,7 @@
       <c r="I11" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -4107,7 +4107,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -4148,7 +4148,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -4189,7 +4189,7 @@
       <c r="I14" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -4271,7 +4271,7 @@
       <c r="I16" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -4312,7 +4312,7 @@
       <c r="I17" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -4353,7 +4353,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -6712,7 +6712,7 @@
       <c r="I9" s="15" t="n">
         <v>34</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+16</t>
         </is>
@@ -6753,7 +6753,7 @@
       <c r="I10" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="40" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -6794,7 +6794,7 @@
       <c r="I11" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -6835,7 +6835,7 @@
       <c r="I12" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -6876,7 +6876,7 @@
       <c r="I13" s="15" t="n">
         <v>31</v>
       </c>
-      <c r="J13" s="40" t="inlineStr">
+      <c r="J13" s="17" t="inlineStr">
         <is>
           <t>+9</t>
         </is>
@@ -6917,7 +6917,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -6958,7 +6958,7 @@
       <c r="I15" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -6999,7 +6999,7 @@
       <c r="I16" s="20" t="n">
         <v>52</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -7040,7 +7040,7 @@
       <c r="I17" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -7081,7 +7081,7 @@
       <c r="I18" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -9440,7 +9440,7 @@
       <c r="I9" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="J9" s="17" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -9481,7 +9481,7 @@
       <c r="I10" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -9522,7 +9522,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -9563,7 +9563,7 @@
       <c r="I12" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -9604,7 +9604,7 @@
       <c r="I13" s="15" t="n">
         <v>73</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -9645,7 +9645,7 @@
       <c r="I14" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -9686,7 +9686,7 @@
       <c r="I15" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -9727,7 +9727,7 @@
       <c r="I16" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -9768,7 +9768,7 @@
       <c r="I17" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-30</t>
         </is>
@@ -9809,7 +9809,7 @@
       <c r="I18" s="20" t="n">
         <v>79</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-33</t>
         </is>
@@ -12168,7 +12168,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="17" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -12209,7 +12209,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -12250,7 +12250,7 @@
       <c r="I11" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -12291,7 +12291,7 @@
       <c r="I12" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -12332,7 +12332,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -12414,7 +12414,7 @@
       <c r="I15" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -12455,7 +12455,7 @@
       <c r="I16" s="20" t="n">
         <v>57</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -12496,7 +12496,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -12537,7 +12537,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -14896,7 +14896,7 @@
       <c r="I9" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J9" s="17" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -14937,7 +14937,7 @@
       <c r="I10" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="40" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
@@ -14978,7 +14978,7 @@
       <c r="I11" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J11" s="40" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -15019,7 +15019,7 @@
       <c r="I12" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -15060,7 +15060,7 @@
       <c r="I13" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -15101,7 +15101,7 @@
       <c r="I14" s="20" t="n">
         <v>60</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -15142,7 +15142,7 @@
       <c r="I15" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -15183,7 +15183,7 @@
       <c r="I16" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -15224,7 +15224,7 @@
       <c r="I17" s="15" t="n">
         <v>61</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -15265,7 +15265,7 @@
       <c r="I18" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 September 2026 om 12:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 September 2026 om 11:50</t>
         </is>
       </c>
     </row>
@@ -15847,9 +15847,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="L6" s="34" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="L6" s="38" t="inlineStr">
+        <is>
+          <t>3-0</t>
         </is>
       </c>
       <c r="M6" s="34" t="inlineStr">
@@ -19520,7 +19520,7 @@
       <c r="I9" s="15" t="n">
         <v>48</v>
       </c>
-      <c r="J9" s="17" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -19561,7 +19561,7 @@
       <c r="I10" s="20" t="n">
         <v>54</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="40" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
@@ -19602,7 +19602,7 @@
       <c r="I11" s="15" t="n">
         <v>38</v>
       </c>
-      <c r="J11" s="40" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>+17</t>
         </is>
@@ -19643,7 +19643,7 @@
       <c r="I12" s="20" t="n">
         <v>42</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -19684,7 +19684,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -19725,7 +19725,7 @@
       <c r="I14" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19766,7 +19766,7 @@
       <c r="I15" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19807,7 +19807,7 @@
       <c r="I16" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -19848,7 +19848,7 @@
       <c r="I17" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-26</t>
         </is>
@@ -19889,7 +19889,7 @@
       <c r="I18" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -22248,7 +22248,7 @@
       <c r="I9" s="15" t="n">
         <v>46</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+7</t>
         </is>
@@ -22289,7 +22289,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22330,7 +22330,7 @@
       <c r="I11" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22371,7 +22371,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="40" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
@@ -22412,7 +22412,7 @@
       <c r="I13" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -22453,7 +22453,7 @@
       <c r="I14" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -22494,7 +22494,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -22535,7 +22535,7 @@
       <c r="I16" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -22576,7 +22576,7 @@
       <c r="I17" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -22617,7 +22617,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -24976,7 +24976,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
@@ -25017,7 +25017,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="40" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
@@ -25058,7 +25058,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25099,7 +25099,7 @@
       <c r="I12" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25140,7 +25140,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -25181,7 +25181,7 @@
       <c r="I14" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -25222,7 +25222,7 @@
       <c r="I15" s="15" t="n">
         <v>69</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -25263,7 +25263,7 @@
       <c r="I16" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -25304,7 +25304,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -25345,7 +25345,7 @@
       <c r="I18" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -27704,7 +27704,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="17" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -27745,7 +27745,7 @@
       <c r="I10" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27786,7 +27786,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -27827,7 +27827,7 @@
       <c r="I12" s="20" t="n">
         <v>54</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="40" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
@@ -27868,7 +27868,7 @@
       <c r="I13" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27909,7 +27909,7 @@
       <c r="I14" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27950,7 +27950,7 @@
       <c r="I15" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -27991,7 +27991,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -28032,7 +28032,7 @@
       <c r="I17" s="15" t="n">
         <v>66</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -28073,7 +28073,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -30432,7 +30432,7 @@
       <c r="I9" s="15" t="n">
         <v>43</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
@@ -30473,7 +30473,7 @@
       <c r="I10" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30514,7 +30514,7 @@
       <c r="I11" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30555,7 +30555,7 @@
       <c r="I12" s="20" t="n">
         <v>70</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -30596,7 +30596,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30637,7 +30637,7 @@
       <c r="I14" s="20" t="n">
         <v>62</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -30678,7 +30678,7 @@
       <c r="I15" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30719,7 +30719,7 @@
       <c r="I16" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -30760,7 +30760,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -30801,7 +30801,7 @@
       <c r="I18" s="20" t="n">
         <v>78</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-36</t>
         </is>
@@ -31264,7 +31264,7 @@
       <c r="I9" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
@@ -31305,7 +31305,7 @@
       <c r="I10" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="40" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
@@ -31346,7 +31346,7 @@
       <c r="I11" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -31387,7 +31387,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -31428,7 +31428,7 @@
       <c r="I13" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -31469,7 +31469,7 @@
       <c r="I14" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -31510,7 +31510,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -31551,7 +31551,7 @@
       <c r="I16" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -31592,7 +31592,7 @@
       <c r="I17" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -31633,7 +31633,7 @@
       <c r="I18" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -36667,7 +36667,7 @@
       <c r="I9" s="15" t="n">
         <v>47</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
@@ -36708,7 +36708,7 @@
       <c r="I10" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="40" t="inlineStr">
         <is>
           <t>+3</t>
         </is>
@@ -36749,7 +36749,7 @@
       <c r="I11" s="15" t="n">
         <v>46</v>
       </c>
-      <c r="J11" s="40" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -36790,7 +36790,7 @@
       <c r="I12" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -36831,7 +36831,7 @@
       <c r="I13" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -36872,7 +36872,7 @@
       <c r="I14" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -36913,7 +36913,7 @@
       <c r="I15" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-25</t>
         </is>
@@ -36954,7 +36954,7 @@
       <c r="I16" s="20" t="n">
         <v>75</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-34</t>
         </is>
@@ -36995,7 +36995,7 @@
       <c r="I17" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -37036,7 +37036,7 @@
       <c r="I18" s="20" t="n">
         <v>73</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39395,7 +39395,7 @@
       <c r="I9" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
@@ -39436,7 +39436,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -39477,7 +39477,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -39518,7 +39518,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -39559,7 +39559,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -39600,7 +39600,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -39641,7 +39641,7 @@
       <c r="I15" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39682,7 +39682,7 @@
       <c r="I16" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -39723,7 +39723,7 @@
       <c r="I17" s="15" t="n">
         <v>71</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-39</t>
         </is>
@@ -39764,7 +39764,7 @@
       <c r="I18" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -42123,7 +42123,7 @@
       <c r="I9" s="15" t="n">
         <v>46</v>
       </c>
-      <c r="J9" s="40" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
@@ -42164,7 +42164,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -42205,7 +42205,7 @@
       <c r="I11" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -42246,7 +42246,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -42287,7 +42287,7 @@
       <c r="I13" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42328,7 +42328,7 @@
       <c r="I14" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42369,7 +42369,7 @@
       <c r="I15" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42410,7 +42410,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -42451,7 +42451,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -42492,7 +42492,7 @@
       <c r="I18" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>-16</t>
         </is>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 21-09-2026 13:45
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 September 2026 om 12:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 September 2026 om 13:45</t>
         </is>
       </c>
     </row>
@@ -986,38 +986,38 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
         <v>7</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>+18</t>
+          <t>+12</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>71%</t>
+          <t>86%</t>
         </is>
       </c>
     </row>
@@ -1027,38 +1027,38 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Feyenoord Rotterdam</t>
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>5</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I4" s="10" t="n">
         <v>7</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>+15</t>
+          <t>+18</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>71%</t>
         </is>
       </c>
     </row>
@@ -1068,11 +1068,11 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>5</v>
@@ -1081,25 +1081,25 @@
         <v>1</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="11" t="n">
         <v>16</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>+11</t>
+          <t>+14</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>71%</t>
         </is>
       </c>
     </row>
@@ -1109,38 +1109,38 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+12</t>
+          <t>+8</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>71%</t>
         </is>
       </c>
     </row>
@@ -1150,38 +1150,38 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>4</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+12</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>57%</t>
         </is>
       </c>
     </row>
@@ -1318,25 +1318,25 @@
         </is>
       </c>
       <c r="C11" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D11" s="16" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H11" s="16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="K11" s="16" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>29%</t>
         </is>
       </c>
     </row>
@@ -1400,25 +1400,25 @@
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>2</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="16" t="n">
         <v>3</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H13" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I13" s="16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J13" s="24" t="inlineStr">
         <is>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="K13" s="16" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>29%</t>
         </is>
       </c>
     </row>
@@ -1437,11 +1437,11 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Telstar 1963</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C14" s="21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" s="21" t="n">
         <v>1</v>
@@ -1450,25 +1450,25 @@
         <v>2</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" s="22" t="n">
         <v>5</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I14" s="21" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J14" s="25" t="inlineStr">
         <is>
-          <t>-6</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>14%</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C15" s="16" t="n">
@@ -1497,10 +1497,10 @@
         <v>5</v>
       </c>
       <c r="H15" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I15" s="16" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="J15" s="24" t="inlineStr">
         <is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 September 2026 om 12:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 September 2026 om 13:45</t>
         </is>
       </c>
     </row>
@@ -15780,9 +15780,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="R5" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="R5" s="40" t="inlineStr">
+        <is>
+          <t>1-0</t>
         </is>
       </c>
       <c r="S5" s="38" t="inlineStr">
@@ -15949,9 +15949,9 @@
           <t>3-1</t>
         </is>
       </c>
-      <c r="M7" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="M7" s="40" t="inlineStr">
+        <is>
+          <t>3-2</t>
         </is>
       </c>
       <c r="N7" s="36" t="inlineStr">
@@ -16113,9 +16113,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="G9" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="G9" s="40" t="inlineStr">
+        <is>
+          <t>5-0</t>
         </is>
       </c>
       <c r="H9" s="35" t="inlineStr">
@@ -16419,9 +16419,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J12" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="J12" s="38" t="inlineStr">
+        <is>
+          <t>1-1</t>
         </is>
       </c>
       <c r="K12" s="35" t="inlineStr">
@@ -33725,21 +33725,21 @@
       </c>
       <c r="B5" s="45" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>+18</t>
+          <t>+12</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
@@ -33855,14 +33855,14 @@
       </c>
       <c r="H8" s="48" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="I8" s="19" t="n">
         <v>1</v>
       </c>
       <c r="J8" s="21" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 22-09-2026 12:27
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 September 2026 om 13:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 September 2026 om 12:27</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 September 2026 om 13:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 September 2026 om 12:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 23-09-2026 12:38
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 September 2026 om 12:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 September 2026 om 12:38</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 September 2026 om 12:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 September 2026 om 12:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 24-09-2026 12:36
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 September 2026 om 12:38</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 September 2026 om 12:36</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 September 2026 om 12:38</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 September 2026 om 12:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 25-09-2026 12:38
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 September 2026 om 12:36</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 September 2026 om 12:38</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 September 2026 om 12:36</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 September 2026 om 12:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 26-09-2026 12:06
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 September 2026 om 12:38</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 September 2026 om 12:06</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 September 2026 om 12:38</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 September 2026 om 12:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 27-09-2026 12:51
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 September 2026 om 12:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 September 2026 om 12:51</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 September 2026 om 12:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 September 2026 om 12:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 28-09-2026 15:06
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 September 2026 om 12:51</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 September 2026 om 15:06</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 September 2026 om 12:51</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 September 2026 om 15:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 29-09-2026 13:51
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 September 2026 om 15:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 September 2026 om 13:51</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 September 2026 om 15:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 September 2026 om 13:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 30-09-2026 13:26
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 September 2026 om 13:51</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 September 2026 om 13:26</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 September 2026 om 13:51</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 September 2026 om 13:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 01-10-2026 14:18
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 September 2026 om 13:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 October 2026 om 14:18</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 September 2026 om 13:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 October 2026 om 14:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 02-10-2026 13:40
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 October 2026 om 14:18</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 October 2026 om 13:40</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 October 2026 om 14:18</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 October 2026 om 13:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 03-10-2026 12:19
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 October 2026 om 13:40</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 October 2026 om 12:19</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 October 2026 om 13:40</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 October 2026 om 12:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 04-10-2026 13:05
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 October 2026 om 12:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 October 2026 om 13:05</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 October 2026 om 12:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 October 2026 om 13:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 05-10-2026 15:40
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 October 2026 om 13:05</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 October 2026 om 15:40</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 October 2026 om 13:05</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 October 2026 om 15:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 06-10-2026 14:00
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 October 2026 om 15:40</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 October 2026 om 14:00</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 October 2026 om 15:40</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 October 2026 om 14:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 07-10-2026 14:18
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 October 2026 om 14:00</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 October 2026 om 14:18</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 October 2026 om 14:00</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 October 2026 om 14:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 08-10-2026 14:27
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 October 2026 om 14:18</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 October 2026 om 14:27</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 October 2026 om 14:18</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 October 2026 om 14:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 09-10-2026 14:13
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 October 2026 om 14:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 October 2026 om 14:13</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 October 2026 om 14:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 October 2026 om 14:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 10-10-2026 13:24
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 October 2026 om 14:13</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 October 2026 om 13:24</t>
         </is>
       </c>
     </row>
@@ -986,11 +986,11 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>6</v>
@@ -999,25 +999,25 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>19</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>+12</t>
+          <t>+16</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>75%</t>
         </is>
       </c>
     </row>
@@ -1027,38 +1027,38 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C4" s="10" t="n">
         <v>7</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>+18</t>
+          <t>+12</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>71%</t>
+          <t>86%</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Feyenoord Rotterdam</t>
         </is>
       </c>
       <c r="C5" s="10" t="n">
@@ -1078,23 +1078,23 @@
         <v>5</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>+18</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
@@ -1359,7 +1359,7 @@
         </is>
       </c>
       <c r="C12" s="21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D12" s="21" t="n">
         <v>2</v>
@@ -1368,7 +1368,7 @@
         <v>3</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12" s="22" t="n">
         <v>9</v>
@@ -1377,16 +1377,16 @@
         <v>11</v>
       </c>
       <c r="I12" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="J12" s="23" t="inlineStr">
-        <is>
-          <t>+2</t>
+        <v>11</v>
+      </c>
+      <c r="J12" s="21" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 October 2026 om 14:13</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 October 2026 om 13:24</t>
         </is>
       </c>
     </row>
@@ -16643,9 +16643,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="P14" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="P14" s="40" t="inlineStr">
+        <is>
+          <t>2-0</t>
         </is>
       </c>
       <c r="Q14" s="40" t="inlineStr">
@@ -33725,21 +33725,21 @@
       </c>
       <c r="B5" s="45" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
         <v>19</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>+12</t>
+          <t>+16</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
@@ -33785,7 +33785,7 @@
         </is>
       </c>
       <c r="I6" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="21" t="n">
         <v>14</v>
@@ -33852,17 +33852,6 @@
         <is>
           <t>+51</t>
         </is>
-      </c>
-      <c r="H8" s="48" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="I8" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="21" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 11-10-2026 13:51
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 October 2026 om 13:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 October 2026 om 13:51</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Feyenoord Rotterdam</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -996,23 +996,23 @@
         <v>6</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>+16</t>
+          <t>+20</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -1027,11 +1027,11 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>6</v>
@@ -1040,25 +1040,25 @@
         <v>1</v>
       </c>
       <c r="F4" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="11" t="n">
         <v>19</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>+12</t>
+          <t>+16</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>75%</t>
         </is>
       </c>
     </row>
@@ -1068,38 +1068,38 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>+18</t>
+          <t>+10</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>71%</t>
+          <t>75%</t>
         </is>
       </c>
     </row>
@@ -1113,25 +1113,25 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>5</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="H6" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="H6" s="10" t="n">
-        <v>15</v>
-      </c>
       <c r="I6" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>71%</t>
+          <t>62%</t>
         </is>
       </c>
     </row>
@@ -1154,25 +1154,25 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>4</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1195,25 +1195,25 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>4</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1273,29 +1273,29 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>FC Groningen</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C10" s="21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" s="22" t="n">
         <v>11</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I10" s="21" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J10" s="23" t="inlineStr">
         <is>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="K10" s="21" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1314,29 +1314,29 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="C11" s="16" t="n">
         <v>7</v>
       </c>
       <c r="D11" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="16" t="n">
-        <v>4</v>
-      </c>
       <c r="F11" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H11" s="16" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="K11" s="16" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>43%</t>
         </is>
       </c>
     </row>
@@ -1400,25 +1400,25 @@
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>2</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="16" t="n">
         <v>3</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H13" s="16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I13" s="16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J13" s="24" t="inlineStr">
         <is>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="K13" s="16" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1437,14 +1437,14 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="C14" s="21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="21" t="n">
         <v>2</v>
@@ -1453,22 +1453,22 @@
         <v>4</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I14" s="21" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="J14" s="25" t="inlineStr">
         <is>
-          <t>-7</t>
+          <t>-11</t>
         </is>
       </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1478,29 +1478,29 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>Telstar 1963</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" s="16" t="n">
         <v>4</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H15" s="16" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="I15" s="16" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J15" s="24" t="inlineStr">
         <is>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="K15" s="16" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>12%</t>
         </is>
       </c>
     </row>
@@ -1519,38 +1519,38 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>SC Cambuur-Leeuwarden</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C16" s="21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D16" s="21" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" s="21" t="n">
         <v>4</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I16" s="21" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J16" s="25" t="inlineStr">
         <is>
-          <t>-9</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="K16" s="21" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>12%</t>
         </is>
       </c>
     </row>
@@ -1560,38 +1560,38 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>FC Utrecht</t>
+          <t>SC Cambuur-Leeuwarden</t>
         </is>
       </c>
       <c r="C17" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D17" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" s="16" t="n">
         <v>4</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H17" s="16" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I17" s="16" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="J17" s="24" t="inlineStr">
         <is>
-          <t>-13</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="K17" s="16" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>12%</t>
         </is>
       </c>
     </row>
@@ -1605,19 +1605,19 @@
         </is>
       </c>
       <c r="C18" s="21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D18" s="21" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="21" t="n">
         <v>5</v>
       </c>
       <c r="G18" s="22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H18" s="21" t="n">
         <v>6</v>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="K18" s="21" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>12%</t>
         </is>
       </c>
     </row>
@@ -1646,25 +1646,25 @@
         </is>
       </c>
       <c r="C19" s="28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D19" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" s="28" t="n">
         <v>5</v>
       </c>
       <c r="G19" s="29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H19" s="28" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I19" s="28" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J19" s="30" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C20" s="28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D20" s="28" t="n">
         <v>0</v>
@@ -1696,20 +1696,20 @@
         <v>2</v>
       </c>
       <c r="F20" s="28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G20" s="29" t="n">
         <v>2</v>
       </c>
       <c r="H20" s="28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I20" s="28" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J20" s="30" t="inlineStr">
         <is>
-          <t>-14</t>
+          <t>-16</t>
         </is>
       </c>
       <c r="K20" s="28" t="inlineStr">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 October 2026 om 13:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 October 2026 om 13:51</t>
         </is>
       </c>
     </row>
@@ -15648,9 +15648,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="K4" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="K4" s="38" t="inlineStr">
+        <is>
+          <t>1-1</t>
         </is>
       </c>
       <c r="L4" s="36" t="inlineStr">
@@ -16076,9 +16076,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="S8" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="S8" s="40" t="inlineStr">
+        <is>
+          <t>3-1</t>
         </is>
       </c>
     </row>
@@ -16098,9 +16098,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="D9" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="D9" s="40" t="inlineStr">
+        <is>
+          <t>2-0</t>
         </is>
       </c>
       <c r="E9" s="36" t="inlineStr">
@@ -16205,9 +16205,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="F10" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>1-1</t>
         </is>
       </c>
       <c r="G10" s="36" t="inlineStr">
@@ -16357,9 +16357,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="Q11" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="Q11" s="38" t="inlineStr">
+        <is>
+          <t>3-3</t>
         </is>
       </c>
       <c r="R11" s="36" t="inlineStr">
@@ -33725,21 +33725,21 @@
       </c>
       <c r="B5" s="45" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Feyenoord Rotterdam</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>+16</t>
+          <t>+20</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
@@ -33785,7 +33785,7 @@
         </is>
       </c>
       <c r="I6" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J6" s="21" t="n">
         <v>14</v>
@@ -33852,6 +33852,17 @@
         <is>
           <t>+51</t>
         </is>
+      </c>
+      <c r="H8" s="48" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 13-10-2026 14:52
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 October 2026 om 16:35</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 October 2026 om 14:52</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 October 2026 om 16:35</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 October 2026 om 14:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 14-10-2026 12:43
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 October 2026 om 14:52</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 October 2026 om 12:43</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 October 2026 om 14:52</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 October 2026 om 12:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 15-10-2026 12:31
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 October 2026 om 12:43</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 October 2026 om 12:31</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 October 2026 om 12:43</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 October 2026 om 12:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 16-10-2026 12:10
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 October 2026 om 12:31</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 October 2026 om 12:10</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 October 2026 om 12:31</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 October 2026 om 12:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 17-10-2026 11:28
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 October 2026 om 12:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 October 2026 om 11:28</t>
         </is>
       </c>
     </row>
@@ -1273,38 +1273,38 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>SC Heerenveen</t>
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G10" s="21" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="I10" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="H10" s="20" t="n">
-        <v>19</v>
-      </c>
-      <c r="I10" s="20" t="n">
-        <v>17</v>
-      </c>
       <c r="J10" s="22" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+4</t>
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -1314,29 +1314,29 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
         <v>8</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11" s="16" t="n">
         <v>11</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J11" s="23" t="inlineStr">
         <is>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1355,38 +1355,38 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>SC Heerenveen</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="20" t="n">
-        <v>3</v>
-      </c>
       <c r="F12" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12" s="21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>11</v>
-      </c>
-      <c r="J12" s="20" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v>18</v>
+      </c>
+      <c r="J12" s="24" t="inlineStr">
+        <is>
+          <t>-2</t>
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 October 2026 om 12:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 October 2026 om 11:28</t>
         </is>
       </c>
     </row>
@@ -16924,9 +16924,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="N17" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="N17" s="39" t="inlineStr">
+        <is>
+          <t>4-0</t>
         </is>
       </c>
       <c r="O17" s="35" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 20-10-2026 12:36
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 October 2026 om 14:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 October 2026 om 12:36</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 October 2026 om 14:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 October 2026 om 12:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 21-10-2026 12:47
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 October 2026 om 12:36</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 October 2026 om 12:47</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 October 2026 om 12:36</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 October 2026 om 12:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 22-10-2026 12:50
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 October 2026 om 12:47</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 October 2026 om 12:50</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 October 2026 om 12:47</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 October 2026 om 12:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 23-10-2026 12:29
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 October 2026 om 12:50</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 October 2026 om 12:29</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 October 2026 om 12:50</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 October 2026 om 12:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 27-10-2026 13:02
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 October 2026 om 14:00</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 October 2026 om 13:02</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 October 2026 om 14:00</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 October 2026 om 13:02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 28-10-2026 13:53
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 October 2026 om 13:02</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 October 2026 om 13:53</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 October 2026 om 13:02</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 October 2026 om 13:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 29-10-2026 13:59
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 October 2026 om 13:53</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 October 2026 om 13:59</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 October 2026 om 13:53</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 October 2026 om 13:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 30-10-2026 13:54
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 October 2026 om 13:59</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 October 2026 om 13:54</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 October 2026 om 13:59</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 October 2026 om 13:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 31-10-2026 13:27
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 October 2026 om 13:54</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  31 October 2026 om 13:27</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 October 2026 om 13:54</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  31 October 2026 om 13:27</t>
         </is>
       </c>
     </row>

</xml_diff>